<commit_message>
Apply professor corrections + VS Code setup for new users
Notebook fixes (MSF_SAAM_Comments.pdf):
- REBALANCE_YEARS: Dec 2013→Dec 2023 (last allocation Dec 2023, not 2024)
- PERF_YEARS: Jan 2014→Dec 2024 (T=132 months, not 144)
- Cumulative return plots: base 1 instead of 100 (all figures)
- Sharpe ratio: explicit RF_ANN=0.0 parameter replacing implicit Rf=0
- Verification checklist: hardcoded 2024→2023 (KeyError fix)
- Report plan updated: all date refs, T=132, performance numbers flagged for recalculation

Setup for new users:
- requirements.txt with all Python dependencies
- README.md rewritten with step-by-step VS Code install guide (Mac/Windows)
- .vscode/extensions.json with recommended extensions (Python + Jupyter)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SAAM_PartI_Results.xlsx
+++ b/SAAM_PartI_Results.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C145"/>
+  <dimension ref="A1:C133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1900,138 +1900,6 @@
       </c>
       <c r="C133" t="n">
         <v>-0.009856214493442898</v>
-      </c>
-    </row>
-    <row r="134">
-      <c r="A134" s="2" t="n">
-        <v>45688</v>
-      </c>
-      <c r="B134" t="n">
-        <v>0.001641557310776805</v>
-      </c>
-      <c r="C134" t="n">
-        <v>0.01459754662739966</v>
-      </c>
-    </row>
-    <row r="135">
-      <c r="A135" s="2" t="n">
-        <v>45716</v>
-      </c>
-      <c r="B135" t="n">
-        <v>0.01907813547572055</v>
-      </c>
-      <c r="C135" t="n">
-        <v>-0.009027104314805703</v>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" s="2" t="n">
-        <v>45747</v>
-      </c>
-      <c r="B136" t="n">
-        <v>0.02650042669169434</v>
-      </c>
-      <c r="C136" t="n">
-        <v>0.003987725657531404</v>
-      </c>
-    </row>
-    <row r="137">
-      <c r="A137" s="2" t="n">
-        <v>45777</v>
-      </c>
-      <c r="B137" t="n">
-        <v>0.04468887585659086</v>
-      </c>
-      <c r="C137" t="n">
-        <v>0.0547894123500869</v>
-      </c>
-    </row>
-    <row r="138">
-      <c r="A138" s="2" t="n">
-        <v>45807</v>
-      </c>
-      <c r="B138" t="n">
-        <v>0.03397091769357879</v>
-      </c>
-      <c r="C138" t="n">
-        <v>0.03867698314236029</v>
-      </c>
-    </row>
-    <row r="139">
-      <c r="A139" s="2" t="n">
-        <v>45838</v>
-      </c>
-      <c r="B139" t="n">
-        <v>0.01763981186037461</v>
-      </c>
-      <c r="C139" t="n">
-        <v>0.02402119631038961</v>
-      </c>
-    </row>
-    <row r="140">
-      <c r="A140" s="2" t="n">
-        <v>45869</v>
-      </c>
-      <c r="B140" t="n">
-        <v>0.00994980280014986</v>
-      </c>
-      <c r="C140" t="n">
-        <v>-0.0001410061433273421</v>
-      </c>
-    </row>
-    <row r="141">
-      <c r="A141" s="2" t="n">
-        <v>45898</v>
-      </c>
-      <c r="B141" t="n">
-        <v>0.06631778629602995</v>
-      </c>
-      <c r="C141" t="n">
-        <v>0.06173830699970397</v>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142" s="2" t="n">
-        <v>45930</v>
-      </c>
-      <c r="B142" t="n">
-        <v>0.01231095441954323</v>
-      </c>
-      <c r="C142" t="n">
-        <v>0.02039728440838235</v>
-      </c>
-    </row>
-    <row r="143">
-      <c r="A143" s="2" t="n">
-        <v>45961</v>
-      </c>
-      <c r="B143" t="n">
-        <v>0.008167842394445041</v>
-      </c>
-      <c r="C143" t="n">
-        <v>0.02823859897027642</v>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" s="2" t="n">
-        <v>45989</v>
-      </c>
-      <c r="B144" t="n">
-        <v>0.02526087059294746</v>
-      </c>
-      <c r="C144" t="n">
-        <v>-0.006507661102928277</v>
-      </c>
-    </row>
-    <row r="145">
-      <c r="A145" s="2" t="n">
-        <v>46022</v>
-      </c>
-      <c r="B145" t="n">
-        <v>-0.006992636251153603</v>
-      </c>
-      <c r="C145" t="n">
-        <v>0.007333753614933499</v>
       </c>
     </row>
   </sheetData>
@@ -2092,13 +1960,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.09809162531292515</v>
+        <v>0.08189881557198686</v>
       </c>
       <c r="C2" t="n">
-        <v>0.1069505587752375</v>
+        <v>0.1089077422040935</v>
       </c>
       <c r="D2" t="n">
-        <v>0.9171679553266298</v>
+        <v>0.75200177613184</v>
       </c>
       <c r="E2" t="n">
         <v>-0.0752445402850781</v>
@@ -2107,7 +1975,7 @@
         <v>0.1036863387621368</v>
       </c>
       <c r="G2" t="n">
-        <v>1.874382698486211</v>
+        <v>1.230263534150617</v>
       </c>
     </row>
     <row r="3">
@@ -2117,13 +1985,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.07744332978873536</v>
+        <v>0.0616561089516201</v>
       </c>
       <c r="C3" t="n">
-        <v>0.1321507554056972</v>
+        <v>0.1353214327477623</v>
       </c>
       <c r="D3" t="n">
-        <v>0.5860226038889269</v>
+        <v>0.4556270776895072</v>
       </c>
       <c r="E3" t="n">
         <v>-0.1144322246260605</v>
@@ -2132,7 +2000,7 @@
         <v>0.1331898733481605</v>
       </c>
       <c r="G3" t="n">
-        <v>1.20663466099004</v>
+        <v>0.7479696278997476</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix annualized return: CAGR formula per professor correction
Switch performance_stats() from arithmetic mean annualized to geometric
CAGR per MSF_SAAM_Comments.pdf slide 4: mu_ann = (1+cum_ret)^(12/T) - 1

Updated Sharpe ratios Jan 2014-Dec 2024 Rf=0: MV 0.695, VW 0.385,
MV50 0.682, VW50 0.391, NZ 0.389. All 5 verification checks pass.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SAAM_PartI_Results.xlsx
+++ b/SAAM_PartI_Results.xlsx
@@ -1960,13 +1960,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.08189881557198686</v>
+        <v>0.07564445797981745</v>
       </c>
       <c r="C2" t="n">
         <v>0.1089077422040935</v>
       </c>
       <c r="D2" t="n">
-        <v>0.75200177613184</v>
+        <v>0.694573741489007</v>
       </c>
       <c r="E2" t="n">
         <v>-0.0752445402850781</v>
@@ -1985,13 +1985,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.0616561089516201</v>
+        <v>0.05207944279674415</v>
       </c>
       <c r="C3" t="n">
         <v>0.1353214327477623</v>
       </c>
       <c r="D3" t="n">
-        <v>0.4556270776895072</v>
+        <v>0.3848573115082197</v>
       </c>
       <c r="E3" t="n">
         <v>-0.1144322246260605</v>

</xml_diff>